<commit_message>
minor adjustments in  chat response for out-of-scope topics
</commit_message>
<xml_diff>
--- a/testset.xlsx
+++ b/testset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dubra\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dubra\Documents\gitRepos\chat-vlscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFA97D0-ECF9-4A0C-87D7-868E542CF8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688E30EE-BAFA-42CA-BD97-D64A33F7121D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="224">
   <si>
     <t>01-introduction.qmd</t>
   </si>
@@ -779,15 +779,6 @@
     <t>Was mache ich wenn zwei Autoren denselben Nachnamen haben?</t>
   </si>
   <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>Ich habe eine Frage bezüglich APA 7-Richtlinien für die Referenzierung im Fliesstext. Ich habe einen Paragraphen, in dem ich eine Studie referenziere. Wie referenziere ich dieselbe Studie im selben paragraphen?</t>
-  </si>
-  <si>
-    <t>Narrative Zitation (Autor im Satz genannt): Wenn du den Autorennamen im Satz integrierst (narrative Referenzierung), musst du das Publikationsjahr nur bei der ersten Nennung im Absatz angeben. Wenn du die Quelle in Klammern angibst, musst du bei jeder Nennung Autor und Jahr vollständig angeben – auch im selben Absatz. Sobald du im Absatz eine andere Quelle nennst oder die Struktur so unklar wird, dass Verwechslungen möglich wären, solltest du das Jahr bei erneuter narrativer Nennung wieder anführen.</t>
-  </si>
-  <si>
     <t>9.3.2 Zitate</t>
   </si>
   <si>
@@ -891,6 +882,12 @@
   </si>
   <si>
     <t>expected_answer</t>
+  </si>
+  <si>
+    <t>8.3 Einleitung &amp; 10.2.1 Einleitung</t>
+  </si>
+  <si>
+    <t>Wie muss man Zahlen runden?</t>
   </si>
 </sst>
 </file>
@@ -928,12 +925,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -948,12 +957,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1289,14 +1300,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4C9E78-AFAD-4E01-BFD3-9EE24F24F280}">
   <dimension ref="A1:D77"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.453125" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" customWidth="1"/>
-    <col min="3" max="3" width="52.1796875" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="32.28515625" customWidth="1"/>
+    <col min="3" max="3" width="52.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1307,15 +1318,15 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -1324,26 +1335,26 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>222</v>
-      </c>
-      <c r="C3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -1352,12 +1363,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -1366,26 +1377,26 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>223</v>
-      </c>
-      <c r="C6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -1394,7 +1405,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1408,12 +1419,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
@@ -1422,7 +1433,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1436,7 +1447,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1450,7 +1461,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1464,7 +1475,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1478,7 +1489,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1492,7 +1503,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1506,7 +1517,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1520,7 +1531,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -1534,7 +1545,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -1548,7 +1559,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -1562,7 +1573,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -1576,7 +1587,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -1587,7 +1598,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -1601,7 +1612,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1615,7 +1626,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -1629,7 +1640,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>42</v>
       </c>
@@ -1643,7 +1654,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -1653,11 +1664,11 @@
       <c r="C26" t="s">
         <v>68</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>67</v>
       </c>
@@ -1667,11 +1678,11 @@
       <c r="C27" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>67</v>
       </c>
@@ -1685,7 +1696,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>67</v>
       </c>
@@ -1699,7 +1710,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>67</v>
       </c>
@@ -1713,7 +1724,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>67</v>
       </c>
@@ -1727,7 +1738,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -1741,7 +1752,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>86</v>
       </c>
@@ -1755,7 +1766,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>90</v>
       </c>
@@ -1769,21 +1780,21 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>90</v>
       </c>
       <c r="B35" t="s">
         <v>93</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="3" t="s">
         <v>94</v>
       </c>
       <c r="D35" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>90</v>
       </c>
@@ -1797,7 +1808,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>90</v>
       </c>
@@ -1811,21 +1822,21 @@
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>90</v>
       </c>
       <c r="B38" t="s">
         <v>100</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="3" t="s">
         <v>101</v>
       </c>
       <c r="D38" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>90</v>
       </c>
@@ -1839,7 +1850,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>106</v>
       </c>
@@ -1853,12 +1864,12 @@
         <v>108</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>106</v>
       </c>
       <c r="B41" t="s">
-        <v>109</v>
+        <v>222</v>
       </c>
       <c r="C41" t="s">
         <v>110</v>
@@ -1867,7 +1878,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>106</v>
       </c>
@@ -1881,7 +1892,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>106</v>
       </c>
@@ -1895,7 +1906,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>106</v>
       </c>
@@ -1909,7 +1920,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>106</v>
       </c>
@@ -1923,7 +1934,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>106</v>
       </c>
@@ -1937,7 +1948,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>106</v>
       </c>
@@ -1951,7 +1962,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>106</v>
       </c>
@@ -1965,7 +1976,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>106</v>
       </c>
@@ -1979,7 +1990,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>106</v>
       </c>
@@ -1993,7 +2004,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>106</v>
       </c>
@@ -2007,7 +2018,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>106</v>
       </c>
@@ -2021,7 +2032,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>106</v>
       </c>
@@ -2035,7 +2046,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>106</v>
       </c>
@@ -2049,7 +2060,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>106</v>
       </c>
@@ -2059,11 +2070,11 @@
       <c r="C55" t="s">
         <v>148</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" s="3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>150</v>
       </c>
@@ -2077,7 +2088,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>150</v>
       </c>
@@ -2087,39 +2098,39 @@
       <c r="C57" t="s">
         <v>156</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="3" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>150</v>
       </c>
       <c r="B58" t="s">
         <v>158</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="3" t="s">
         <v>159</v>
       </c>
       <c r="D58" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>150</v>
       </c>
       <c r="B59" t="s">
-        <v>166</v>
-      </c>
-      <c r="C59" t="s">
-        <v>163</v>
+        <v>158</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>223</v>
       </c>
       <c r="D59" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>150</v>
       </c>
@@ -2127,97 +2138,97 @@
         <v>166</v>
       </c>
       <c r="C60" t="s">
-        <v>164</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+      <c r="D60" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>150</v>
       </c>
       <c r="B61" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C61" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D61" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>150</v>
       </c>
       <c r="B62" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C62" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D62" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>150</v>
       </c>
       <c r="B63" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C63" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D63" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>150</v>
       </c>
       <c r="B64" t="s">
-        <v>176</v>
-      </c>
-      <c r="C64" t="s">
-        <v>178</v>
-      </c>
-      <c r="D64" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>150</v>
       </c>
       <c r="B65" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C65" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D65" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>150</v>
       </c>
       <c r="B66" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C66" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D66" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>150</v>
       </c>
@@ -2225,150 +2236,150 @@
         <v>184</v>
       </c>
       <c r="C67" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D67" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>150</v>
       </c>
       <c r="B68" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C68" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D68" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>150</v>
       </c>
       <c r="B69" t="s">
+        <v>187</v>
+      </c>
+      <c r="C69" t="s">
+        <v>188</v>
+      </c>
+      <c r="D69" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>150</v>
+      </c>
+      <c r="B70" t="s">
+        <v>190</v>
+      </c>
+      <c r="C70" t="s">
+        <v>191</v>
+      </c>
+      <c r="D70" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>196</v>
+      </c>
+      <c r="B71" t="s">
+        <v>195</v>
+      </c>
+      <c r="C71" t="s">
+        <v>194</v>
+      </c>
+      <c r="D71" t="s">
         <v>193</v>
       </c>
-      <c r="C69" t="s">
-        <v>194</v>
-      </c>
-      <c r="D69" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>196</v>
+      </c>
+      <c r="B72" t="s">
         <v>199</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C72" t="s">
         <v>198</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D72" t="s">
         <v>197</v>
       </c>
-      <c r="D70" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>199</v>
-      </c>
-      <c r="B71" t="s">
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>204</v>
+      </c>
+      <c r="B73" t="s">
+        <v>203</v>
+      </c>
+      <c r="C73" t="s">
+        <v>201</v>
+      </c>
+      <c r="D73" t="s">
         <v>202</v>
       </c>
-      <c r="C71" t="s">
-        <v>201</v>
-      </c>
-      <c r="D71" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>207</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B74" t="s">
+        <v>208</v>
+      </c>
+      <c r="C74" t="s">
+        <v>205</v>
+      </c>
+      <c r="D74" t="s">
         <v>206</v>
       </c>
-      <c r="C72" t="s">
-        <v>204</v>
-      </c>
-      <c r="D72" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>209</v>
+      </c>
+      <c r="B75" t="s">
+        <v>212</v>
+      </c>
+      <c r="C75" t="s">
         <v>210</v>
       </c>
-      <c r="B73" t="s">
+      <c r="D75" t="s">
         <v>211</v>
       </c>
-      <c r="C73" t="s">
-        <v>208</v>
-      </c>
-      <c r="D73" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>212</v>
-      </c>
-      <c r="B74" t="s">
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>216</v>
+      </c>
+      <c r="B76" t="s">
         <v>215</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C76" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D76" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>219</v>
-      </c>
-      <c r="B75" t="s">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>216</v>
+      </c>
+      <c r="B77" t="s">
+        <v>215</v>
+      </c>
+      <c r="C77" t="s">
+        <v>217</v>
+      </c>
+      <c r="D77" t="s">
         <v>218</v>
-      </c>
-      <c r="C75" t="s">
-        <v>216</v>
-      </c>
-      <c r="D75" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>219</v>
-      </c>
-      <c r="B76" t="s">
-        <v>218</v>
-      </c>
-      <c r="C76" t="s">
-        <v>220</v>
-      </c>
-      <c r="D76" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>187</v>
-      </c>
-      <c r="B77" t="s">
-        <v>187</v>
-      </c>
-      <c r="C77" t="s">
-        <v>188</v>
-      </c>
-      <c r="D77" t="s">
-        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add weblinks to poster examples
</commit_message>
<xml_diff>
--- a/testset.xlsx
+++ b/testset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dubra\Documents\gitRepos\chat-vlscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA3ABB4-C47C-4805-ACA9-AB35E27D01A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D514E1F6-9BAD-4509-A034-38DF89880E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="230">
   <si>
     <t>01-introduction.qmd</t>
   </si>
@@ -897,6 +897,15 @@
   </si>
   <si>
     <t>14.1 Inhalte eines Posters</t>
+  </si>
+  <si>
+    <t>Gib mire ein paar Posterbeispiele</t>
+  </si>
+  <si>
+    <t>14.5 Posterbeispiele</t>
+  </si>
+  <si>
+    <t>Nachfolgend werden einige Beispiele von Postern aufgeführt inkl. Weblinks zu den Postern.</t>
   </si>
 </sst>
 </file>
@@ -1307,7 +1316,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4C9E78-AFAD-4E01-BFD3-9EE24F24F280}">
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" customWidth="1"/>
@@ -2404,6 +2413,20 @@
         <v>218</v>
       </c>
     </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>216</v>
+      </c>
+      <c r="B79" t="s">
+        <v>228</v>
+      </c>
+      <c r="C79" t="s">
+        <v>227</v>
+      </c>
+      <c r="D79" t="s">
+        <v>229</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactoring utils for evaluation
</commit_message>
<xml_diff>
--- a/testset.xlsx
+++ b/testset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dubra\Documents\gitRepos\chat-vlscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9310E3C-FE25-4E39-9777-58377E3FCF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0905D280-FB24-4965-9177-5BCCAFCEEE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="231">
   <si>
     <t>01-introduction.qmd</t>
   </si>
@@ -906,6 +906,9 @@
   </si>
   <si>
     <t>Gib mir ein paar Posterbeispiele</t>
+  </si>
+  <si>
+    <t>id</t>
   </si>
 </sst>
 </file>
@@ -1316,1114 +1319,1351 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4C9E78-AFAD-4E01-BFD3-9EE24F24F280}">
-  <dimension ref="A1:D79"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E79"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" customWidth="1"/>
-    <col min="3" max="3" width="52.140625" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" customWidth="1"/>
+    <col min="3" max="3" width="32.26953125" customWidth="1"/>
+    <col min="4" max="4" width="52.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>219</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>219</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>219</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>220</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>220</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>220</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>134</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>200</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>19</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>24</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>27</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>30</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>33</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>35</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>37</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>41</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>39</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
         <v>42</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>43</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>44</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
         <v>42</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>45</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>46</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
         <v>42</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>49</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>48</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
         <v>42</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>51</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>52</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>42</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>55</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>58</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>56</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
         <v>42</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>61</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>60</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
         <v>42</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>61</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>62</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
         <v>42</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>66</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>64</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
         <v>67</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>124</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>68</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
         <v>67</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>70</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>71</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
         <v>67</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>77</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>73</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
         <v>67</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>77</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>75</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
         <v>67</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>77</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>78</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
         <v>67</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>80</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>81</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
         <v>67</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>83</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>84</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
         <v>86</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>89</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>87</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
         <v>90</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>154</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>91</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
         <v>90</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="D35" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
         <v>90</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>96</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>99</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
         <v>90</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>96</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>97</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
         <v>90</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>100</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="D38" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
         <v>90</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>103</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>104</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
         <v>106</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>155</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>107</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
         <v>106</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
         <v>222</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>110</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
         <v>106</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>109</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>111</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
         <v>106</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>109</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>113</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
         <v>106</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>115</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>116</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
         <v>106</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>115</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>118</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
         <v>106</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>115</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>121</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
         <v>106</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>123</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>125</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
         <v>106</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>127</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>128</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
         <v>106</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>127</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>130</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
         <v>106</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>161</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>132</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
         <v>106</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>135</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>138</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
         <v>106</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>136</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>139</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
         <v>106</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>143</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>142</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
         <v>106</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>144</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>145</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
         <v>106</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>147</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>148</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="E55" s="3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
         <v>150</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>153</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>151</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
         <v>150</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>158</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>156</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="E57" s="3" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
         <v>150</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>158</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="D58" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
         <v>150</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>158</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
         <v>223</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
         <v>150</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>166</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>163</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
         <v>150</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>166</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
         <v>164</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
         <v>150</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>170</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>168</v>
       </c>
-      <c r="D62" t="s">
+      <c r="E62" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
         <v>150</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
         <v>169</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>171</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
         <v>150</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>175</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="D64" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="E64" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
         <v>150</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
         <v>176</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>178</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
         <v>150</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>181</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>179</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
         <v>150</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>184</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>182</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
         <v>150</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>184</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>186</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
         <v>150</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>187</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>188</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
         <v>150</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>190</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>191</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
         <v>196</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>195</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>194</v>
       </c>
-      <c r="D71" t="s">
+      <c r="E71" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
         <v>196</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>199</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>198</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
         <v>204</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>203</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>201</v>
       </c>
-      <c r="D73" t="s">
+      <c r="E73" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
         <v>207</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>208</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>205</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
         <v>209</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>212</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>210</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
         <v>216</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>226</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="D76" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="D76" s="2" t="s">
+      <c r="E76" s="2" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
         <v>216</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>215</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="D77" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D77" s="2" t="s">
+      <c r="E77" s="2" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
         <v>216</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>215</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>217</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
         <v>216</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C79" t="s">
         <v>227</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>229</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="E79" s="2" t="s">
         <v>228</v>
       </c>
     </row>

</xml_diff>

<commit_message>
weblinks added and new embeddings generated, evaluation improved, readme adjusted, experimented with TF-IDF
</commit_message>
<xml_diff>
--- a/testset.xlsx
+++ b/testset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dubra\Documents\gitRepos\chat-vlscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0905D280-FB24-4965-9177-5BCCAFCEEE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D2A7F2-6C2B-4D68-B41E-DE6E0C1EB795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="245">
   <si>
     <t>01-introduction.qmd</t>
   </si>
@@ -386,18 +386,12 @@
     <t>Bei der Präregistriereung werden die Theorie, die davon abgeleiteten Hypothesen, Methoden und Datenanalyse vor dem Beginn der Datenerhebung schriftlich festgehalten und mit Zeitstempel «eingefroren», so dass diese nicht im Nachhinein noch verändert werden können.</t>
   </si>
   <si>
-    <t>06-manuscript.qmd</t>
-  </si>
-  <si>
     <t>Wo sind die Richtlinien für die erstellung von Manuskripten nachzulesen?</t>
   </si>
   <si>
     <t>Für die Psychologie werden diese Konventionen im Publikationsmanual der Amerikanischen Psychologischen Gesellschaft definiert</t>
   </si>
   <si>
-    <t>6 Manuskript</t>
-  </si>
-  <si>
     <t>07-structure.qmd</t>
   </si>
   <si>
@@ -426,9 +420,6 @@
   </si>
   <si>
     <t>Was ist bei einem Paragraphen zu beachten?</t>
-  </si>
-  <si>
-    <t>7.4 Struktur eines Satzes</t>
   </si>
   <si>
     <t>Defizit im deklarativen Gedächtnis</t>
@@ -884,9 +875,6 @@
     <t>expected_answer</t>
   </si>
   <si>
-    <t>8.3 Einleitung &amp; 10.2.1 Einleitung</t>
-  </si>
-  <si>
     <t>Wie muss man Zahlen runden?</t>
   </si>
   <si>
@@ -909,6 +897,60 @@
   </si>
   <si>
     <t>id</t>
+  </si>
+  <si>
+    <t>03-literature.qmd, 08-content.qmd</t>
+  </si>
+  <si>
+    <t>03-literature.qmd, 08-content.qmd, 11-cycle.qmd</t>
+  </si>
+  <si>
+    <t>05-dataanalysis.qmd, 08-content.qmd</t>
+  </si>
+  <si>
+    <t>07-structure.qmd, 09-formatting.qmd</t>
+  </si>
+  <si>
+    <t>08-content.qmd, 09-formatting.qmd</t>
+  </si>
+  <si>
+    <t>8.3 Einleitung &amp; 7.1 Struktur des Manuskriptes (siehe Tabelle) &amp; 7.2 Struktur der Hauptteile &amp; 10.2.1 Einleitung</t>
+  </si>
+  <si>
+    <t>08-content.qmd, 07-structure.html, 10-writing.qmd</t>
+  </si>
+  <si>
+    <t>9  Formatierung des Manuskripts Vorlage</t>
+  </si>
+  <si>
+    <t>Hast du eine Manuskript Vorlage für mich?</t>
+  </si>
+  <si>
+    <t>Um die Arbeit bei der Manuskriptgestaltung zu vereinfachen, wurde eine Vorlage vorbereitet. Die Vorlage ist gemäss den formalen Richtlinien der APA formatiert. Es muss nur noch der Inhalt entsprechend dem Experiment ersetzt werden. Um die Formatierung braucht man sich nicht mehr kümmern.</t>
+  </si>
+  <si>
+    <t>7.4 Struktur eines Satzes (siehe Tabelle)</t>
+  </si>
+  <si>
+    <t>13.4 Beispiele von Vorträgen</t>
+  </si>
+  <si>
+    <t>Nachfolgend werden einige Beispiele von Vorträgen aufgeführt. [links] zu vorträgen</t>
+  </si>
+  <si>
+    <t>Gib mir ein paar Beispiele für gute Vorträge.</t>
+  </si>
+  <si>
+    <t>6 Manuskript &amp; 9.1 Allgemeine Richtlinien</t>
+  </si>
+  <si>
+    <t>06-manuscript.qmd, 09-formatting.qmd</t>
+  </si>
+  <si>
+    <t>Kannst du mir das APA template geben?</t>
+  </si>
+  <si>
+    <t>Ja, natürlich! Hier ist der Link zur Vorlage im APA-Format für die Manuskriptgestaltung: APA7 Vorlage</t>
   </si>
 </sst>
 </file>
@@ -1319,17 +1361,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A4C9E78-AFAD-4E01-BFD3-9EE24F24F280}">
-  <dimension ref="A1:E79"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E82"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.453125" customWidth="1"/>
-    <col min="3" max="3" width="32.26953125" customWidth="1"/>
-    <col min="4" max="4" width="52.1796875" customWidth="1"/>
+    <col min="2" max="2" width="84.42578125" customWidth="1"/>
+    <col min="3" max="3" width="96.5703125" customWidth="1"/>
+    <col min="4" max="4" width="52.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1341,10 +1383,10 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1352,7 +1394,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>
@@ -1361,7 +1403,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1369,7 +1411,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
@@ -1378,7 +1420,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1386,7 +1428,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -1395,7 +1437,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1403,7 +1445,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D5" t="s">
         <v>9</v>
@@ -1412,7 +1454,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1420,7 +1462,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -1429,7 +1471,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1437,7 +1479,7 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -1446,15 +1488,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>227</v>
       </c>
       <c r="C8" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -1463,15 +1505,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>228</v>
       </c>
       <c r="C9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D9" t="s">
         <v>19</v>
@@ -1480,7 +1522,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1497,7 +1539,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1514,7 +1556,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1531,7 +1573,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1548,7 +1590,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1565,7 +1607,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1582,7 +1624,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1599,7 +1641,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1613,10 +1655,10 @@
         <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1633,7 +1675,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1650,7 +1692,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1667,7 +1709,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1681,7 +1723,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1698,7 +1740,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1715,7 +1757,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1732,7 +1774,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1749,15 +1791,15 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>229</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D26" t="s">
         <v>68</v>
@@ -1766,7 +1808,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1783,7 +1825,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1800,7 +1842,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1817,7 +1859,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1834,7 +1876,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1851,7 +1893,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1868,803 +1910,854 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>242</v>
+      </c>
+      <c r="C33" t="s">
+        <v>241</v>
+      </c>
+      <c r="D33" t="s">
         <v>86</v>
       </c>
-      <c r="C33" t="s">
-        <v>89</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>87</v>
       </c>
-      <c r="E33" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>230</v>
+      </c>
+      <c r="C34" t="s">
+        <v>151</v>
+      </c>
+      <c r="D34" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" t="s">
         <v>90</v>
       </c>
-      <c r="C34" t="s">
-        <v>154</v>
-      </c>
-      <c r="D34" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C35" t="s">
+        <v>91</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E35" t="s">
         <v>93</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E35" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C36" t="s">
+        <v>94</v>
+      </c>
+      <c r="D36" t="s">
+        <v>97</v>
+      </c>
+      <c r="E36" t="s">
         <v>96</v>
       </c>
-      <c r="D36" t="s">
-        <v>99</v>
-      </c>
-      <c r="E36" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C37" t="s">
+        <v>94</v>
+      </c>
+      <c r="D37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E37" t="s">
         <v>96</v>
       </c>
-      <c r="D37" t="s">
-        <v>97</v>
-      </c>
-      <c r="E37" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C38" t="s">
-        <v>100</v>
+        <v>237</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E38" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D39" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E39" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>106</v>
+        <v>231</v>
       </c>
       <c r="C40" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D40" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E40" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>106</v>
+        <v>233</v>
       </c>
       <c r="C41" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="D41" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E41" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>106</v>
+        <v>233</v>
       </c>
       <c r="C42" t="s">
+        <v>232</v>
+      </c>
+      <c r="D42" t="s">
+        <v>108</v>
+      </c>
+      <c r="E42" t="s">
         <v>109</v>
       </c>
-      <c r="D42" t="s">
-        <v>111</v>
-      </c>
-      <c r="E42" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" t="s">
         <v>106</v>
       </c>
-      <c r="C43" t="s">
-        <v>109</v>
-      </c>
       <c r="D43" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E43" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D44" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E44" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C45" t="s">
+        <v>112</v>
+      </c>
+      <c r="D45" t="s">
         <v>115</v>
       </c>
-      <c r="D45" t="s">
-        <v>118</v>
-      </c>
       <c r="E45" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C46" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D46" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E46" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C47" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47" t="s">
+        <v>122</v>
+      </c>
+      <c r="E47" t="s">
         <v>123</v>
       </c>
-      <c r="D47" t="s">
-        <v>125</v>
-      </c>
-      <c r="E47" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C48" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D48" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C49" t="s">
+        <v>124</v>
+      </c>
+      <c r="D49" t="s">
         <v>127</v>
       </c>
-      <c r="D49" t="s">
-        <v>130</v>
-      </c>
       <c r="E49" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>231</v>
       </c>
       <c r="C50" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D50" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E50" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C51" t="s">
+        <v>132</v>
+      </c>
+      <c r="D51" t="s">
         <v>135</v>
       </c>
-      <c r="D51" t="s">
-        <v>138</v>
-      </c>
       <c r="E51" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C52" t="s">
+        <v>133</v>
+      </c>
+      <c r="D52" t="s">
         <v>136</v>
       </c>
-      <c r="D52" t="s">
-        <v>139</v>
-      </c>
       <c r="E52" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C53" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D53" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E53" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C54" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D54" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E54" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C55" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D55" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>147</v>
+      </c>
+      <c r="C56" t="s">
         <v>150</v>
       </c>
-      <c r="C56" t="s">
-        <v>153</v>
-      </c>
       <c r="D56" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E56" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C57" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D57" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C58" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E58" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D59" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="E59" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C60" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D60" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E60" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C61" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D61" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E61" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C62" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D62" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E62" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C63" t="s">
+        <v>166</v>
+      </c>
+      <c r="D63" t="s">
+        <v>168</v>
+      </c>
+      <c r="E63" t="s">
         <v>169</v>
       </c>
-      <c r="D63" t="s">
-        <v>171</v>
-      </c>
-      <c r="E63" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C64" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C65" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D65" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E65" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C66" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D66" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E66" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C67" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D67" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E67" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C68" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D68" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E68" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C69" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D69" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E69" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C70" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D70" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E70" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>196</v>
+        <v>147</v>
       </c>
       <c r="C71" t="s">
-        <v>195</v>
-      </c>
-      <c r="D71" t="s">
-        <v>194</v>
-      </c>
-      <c r="E71" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>196</v>
+        <v>147</v>
       </c>
       <c r="C72" t="s">
-        <v>199</v>
-      </c>
-      <c r="D72" t="s">
-        <v>198</v>
-      </c>
-      <c r="E72" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="C73" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="D73" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="E73" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="C74" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="D74" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="E74" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C75" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="D75" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="E75" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="C76" t="s">
-        <v>226</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+      <c r="D76" t="s">
+        <v>202</v>
+      </c>
+      <c r="E76" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="C77" t="s">
-        <v>215</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+        <v>209</v>
+      </c>
+      <c r="D77" t="s">
+        <v>207</v>
+      </c>
+      <c r="E77" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="C78" t="s">
-        <v>215</v>
+        <v>238</v>
       </c>
       <c r="D78" t="s">
-        <v>217</v>
+        <v>240</v>
       </c>
       <c r="E78" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C79" t="s">
-        <v>227</v>
-      </c>
-      <c r="D79" t="s">
-        <v>229</v>
+        <v>222</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>220</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>213</v>
+      </c>
+      <c r="C80" t="s">
+        <v>212</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>213</v>
+      </c>
+      <c r="C81" t="s">
+        <v>212</v>
+      </c>
+      <c r="D81" t="s">
+        <v>214</v>
+      </c>
+      <c r="E81" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>213</v>
+      </c>
+      <c r="C82" t="s">
+        <v>223</v>
+      </c>
+      <c r="D82" t="s">
+        <v>225</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hybrid search evaluation & documentation, testset corrected
</commit_message>
<xml_diff>
--- a/testset.xlsx
+++ b/testset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dubra\Documents\gitRepos\chat-vlscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D2A7F2-6C2B-4D68-B41E-DE6E0C1EB795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC04BCD6-9598-4364-B135-1A4939B3CA71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{85DC4CA6-13D9-4DA1-A147-A77570202D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -917,9 +917,6 @@
     <t>8.3 Einleitung &amp; 7.1 Struktur des Manuskriptes (siehe Tabelle) &amp; 7.2 Struktur der Hauptteile &amp; 10.2.1 Einleitung</t>
   </si>
   <si>
-    <t>08-content.qmd, 07-structure.html, 10-writing.qmd</t>
-  </si>
-  <si>
     <t>9  Formatierung des Manuskripts Vorlage</t>
   </si>
   <si>
@@ -951,6 +948,9 @@
   </si>
   <si>
     <t>Ja, natürlich! Hier ist der Link zur Vorlage im APA-Format für die Manuskriptgestaltung: APA7 Vorlage</t>
+  </si>
+  <si>
+    <t>08-content.qmd, 07-structure.qmd, 10-writing.qmd</t>
   </si>
 </sst>
 </file>
@@ -1915,10 +1915,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C33" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D33" t="s">
         <v>86</v>
@@ -2003,7 +2003,7 @@
         <v>88</v>
       </c>
       <c r="C38" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>98</v>
@@ -2051,7 +2051,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="C41" t="s">
         <v>232</v>
@@ -2068,7 +2068,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="C42" t="s">
         <v>232</v>
@@ -2564,13 +2564,13 @@
         <v>147</v>
       </c>
       <c r="C71" t="s">
+        <v>233</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D71" s="2" t="s">
+      <c r="E71" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -2581,13 +2581,13 @@
         <v>147</v>
       </c>
       <c r="C72" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D72" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E72" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -2683,13 +2683,13 @@
         <v>206</v>
       </c>
       <c r="C78" t="s">
+        <v>237</v>
+      </c>
+      <c r="D78" t="s">
+        <v>239</v>
+      </c>
+      <c r="E78" t="s">
         <v>238</v>
-      </c>
-      <c r="D78" t="s">
-        <v>240</v>
-      </c>
-      <c r="E78" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>